<commit_message>
feat: add new evaluation tasks and update assets for LibreOffice, Inkscape, Kdenlive, Blender domains
- Add 30+ new task JSONs for libreoffice_impr_njc, libreoffice_calc_njc, libreoffice_writ_njc, kdenlive, blender, inkscape
- Add backup_json directory and example_final task configs
- Update LibreOffice Calc/Impress/Writer asset files (.xlsx, .pptx, .docx)
- Add libreoffice_suite_njc task examples and windows evaluator config
- Update taiji_task scripts (r3agentv3, interactive, vllm)
- Add test scripts: test_thinking_mode.py, test_user_model.py, check_task_coverage.py
- Remove deprecated evaluation list JSONs (gimp_new, inkscape_all, kdenlive_all, etc.)
- Update example_final_interactive_all and example_final_non_interactive_all task lists

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/libreoffice_calc_njc/2364b616-c254-40d2-ac46-29b63af72326/InvRestock_L3_08.xlsx
+++ b/assets/libreoffice_calc_njc/2364b616-c254-40d2-ac46-29b63af72326/InvRestock_L3_08.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="57">
   <si>
     <t xml:space="preserve">SKU</t>
   </si>
@@ -175,6 +175,15 @@
   </si>
   <si>
     <t xml:space="preserve">Items to Restock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Restock Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TechGlobal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TechPro</t>
   </si>
   <si>
     <t xml:space="preserve">Items</t>
@@ -268,7 +277,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -282,6 +291,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -320,7 +333,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J16"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="8.53"/>
@@ -359,25 +372,25 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="1" t="n">
@@ -394,25 +407,25 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="4" t="s">
         <v>13</v>
       </c>
       <c r="H3" s="1" t="n">
@@ -429,25 +442,25 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="1" t="n">
@@ -464,25 +477,25 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H5" s="1" t="n">
@@ -499,25 +512,25 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="4" t="n">
         <v>150</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H6" s="1" t="n">
@@ -534,25 +547,25 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H7" s="1" t="n">
@@ -569,25 +582,25 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H8" s="1" t="n">
@@ -604,25 +617,25 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H9" s="1" t="n">
@@ -639,25 +652,25 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="4" t="n">
         <v>89.99</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" s="4" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="1" t="n">
@@ -674,25 +687,25 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="4" t="n">
         <v>899.99</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H11" s="1" t="n">
@@ -709,25 +722,25 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="E12" s="0" t="n">
+      <c r="E12" s="4" t="n">
         <v>449.99</v>
       </c>
-      <c r="F12" s="0" t="n">
+      <c r="F12" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="G12" s="4" t="s">
         <v>39</v>
       </c>
       <c r="H12" s="1" t="n">
@@ -744,25 +757,25 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="E13" s="0" t="n">
+      <c r="E13" s="4" t="n">
         <v>599.99</v>
       </c>
-      <c r="F13" s="0" t="n">
+      <c r="F13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="G13" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H13" s="1" t="n">
@@ -779,25 +792,25 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="E14" s="0" t="n">
+      <c r="E14" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F14" s="0" t="n">
+      <c r="F14" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="G14" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H14" s="1" t="n">
@@ -814,25 +827,25 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="0" t="n">
+      <c r="D15" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="E15" s="0" t="n">
+      <c r="E15" s="4" t="n">
         <v>34.99</v>
       </c>
-      <c r="F15" s="0" t="n">
+      <c r="F15" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="0" t="s">
+      <c r="G15" s="4" t="s">
         <v>47</v>
       </c>
       <c r="H15" s="1" t="n">
@@ -849,25 +862,25 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="0" t="n">
+      <c r="D16" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="E16" s="0" t="n">
+      <c r="E16" s="4" t="n">
         <v>59.99</v>
       </c>
-      <c r="F16" s="0" t="n">
+      <c r="F16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" s="4" t="s">
         <v>47</v>
       </c>
       <c r="H16" s="1" t="n">
@@ -899,15 +912,51 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="4" t="s">
         <v>50</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <f aca="false">SUMIF(Inventory!$G:$G,A2,Inventory!$J:$J)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <f aca="false">SUMIF(Inventory!$G:$G,A3,Inventory!$J:$J)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <f aca="false">SUMIF(Inventory!$G:$G,A4,Inventory!$J:$J)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -927,99 +976,99 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" s="0" t="s">
-        <v>52</v>
+      <c r="B1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="4" t="n">
         <v>1240</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>37839.6</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="4" t="n">
         <v>280</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>28397.2</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="4" t="n">
         <v>190</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>75298.1</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="4" t="n">
         <v>115</v>
       </c>
       <c r="D5" s="1" t="n">

</xml_diff>

<commit_message>
feat: add Kimi/Qwen3.5VL agents, fix duplicate task IDs in interactive eval list, improve stats script
- Add Kimi K2.5 agent (mm_agents/kimi/) and run script (run_multienv_kimi_k25.py)
- Add Qwen3.5-VL agent (mm_agents/qwen35vl_agent.py) and run script (run_multienv_qwen35vl.py)
- Add corresponding taiji launch scripts for Kimi and Qwen3.5
- Fix example_final_interactive_all.json: remove 19 duplicate task IDs (ui_gen domain removed, L3_interactive_inkscape_correction_001 deduped from interactive_xt)
- Fix stats_result_by_software_and_level.py: add libreoffice_multi_njc and multiapp aliases so interactive_multiapp_* tasks are counted correctly
- Update lib_run_single.py, lib_run_interactive.py, taiji start scripts
- Update LibreOffice calc/impr/writ asset files

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/libreoffice_calc_njc/2364b616-c254-40d2-ac46-29b63af72326/InvRestock_L3_08.xlsx
+++ b/assets/libreoffice_calc_njc/2364b616-c254-40d2-ac46-29b63af72326/InvRestock_L3_08.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId2"/>
@@ -203,7 +203,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -225,14 +225,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -277,7 +269,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -286,15 +278,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -372,25 +360,25 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="2" t="n">
         <v>12.99</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="1" t="n">
@@ -407,25 +395,25 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="2" t="n">
         <v>29.99</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H3" s="1" t="n">
@@ -442,25 +430,25 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="2" t="n">
         <v>79.99</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="1" t="n">
@@ -477,25 +465,25 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="2" t="n">
         <v>14.99</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H5" s="1" t="n">
@@ -512,25 +500,25 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="2" t="n">
         <v>39.99</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H6" s="1" t="n">
@@ -547,25 +535,25 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="2" t="n">
         <v>24.99</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H7" s="1" t="n">
@@ -582,25 +570,25 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="2" t="n">
         <v>49.99</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="2" t="s">
         <v>28</v>
       </c>
       <c r="H8" s="1" t="n">
@@ -617,25 +605,25 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="2" t="n">
         <v>149.99</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="2" t="s">
         <v>28</v>
       </c>
       <c r="H9" s="1" t="n">
@@ -652,25 +640,25 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="2" t="n">
         <v>89.99</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="2" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="1" t="n">
@@ -687,25 +675,25 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="2" t="n">
         <v>899.99</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H11" s="1" t="n">
@@ -722,25 +710,25 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="2" t="n">
         <v>449.99</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="F12" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="2" t="s">
         <v>39</v>
       </c>
       <c r="H12" s="1" t="n">
@@ -757,25 +745,25 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="2" t="n">
         <v>599.99</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H13" s="1" t="n">
@@ -792,25 +780,25 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="2" t="n">
         <v>69.99</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="F14" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="2" t="s">
         <v>36</v>
       </c>
       <c r="H14" s="1" t="n">
@@ -827,25 +815,25 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="2" t="s">
         <v>47</v>
       </c>
       <c r="H15" s="1" t="n">
@@ -862,25 +850,25 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="2" t="n">
         <v>59.99</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="2" t="s">
         <v>47</v>
       </c>
       <c r="H16" s="1" t="n">
@@ -913,49 +901,52 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="4" t="n">
-        <v>2</v>
+      <c r="B2" s="2" t="n">
+        <f aca="false">COUNTIFS(Inventory!$G:$G,A2,Inventory!$I:$I,"&gt;0")</f>
+        <v>0</v>
       </c>
       <c r="C2" s="1" t="n">
-        <f aca="false">SUMIF(Inventory!$G:$G,A2,Inventory!$J:$J)</f>
+        <f aca="false">ROUND(SUMIF(Inventory!$G:$G,A2,Inventory!$J:$J),2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>1</v>
+      <c r="B3" s="2" t="n">
+        <f aca="false">COUNTIFS(Inventory!$G:$G,A3,Inventory!$I:$I,"&gt;0")</f>
+        <v>0</v>
       </c>
       <c r="C3" s="1" t="n">
-        <f aca="false">SUMIF(Inventory!$G:$G,A3,Inventory!$J:$J)</f>
+        <f aca="false">ROUND(SUMIF(Inventory!$G:$G,A3,Inventory!$J:$J),2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>3</v>
+      <c r="B4" s="2" t="n">
+        <f aca="false">COUNTIFS(Inventory!$G:$G,A4,Inventory!$I:$I,"&gt;0")</f>
+        <v>0</v>
       </c>
       <c r="C4" s="1" t="n">
-        <f aca="false">SUMIF(Inventory!$G:$G,A4,Inventory!$J:$J)</f>
+        <f aca="false">ROUND(SUMIF(Inventory!$G:$G,A4,Inventory!$J:$J),2)</f>
         <v>0</v>
       </c>
     </row>
@@ -976,19 +967,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1002,82 +993,102 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="2" t="n">
+        <f aca="false">COUNTIF(Inventory!$C:$C,A2)</f>
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="2" t="n">
+        <f aca="false">SUMIF(Inventory!$C:$C,A2,Inventory!$D:$D)</f>
         <v>1240</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>37839.6</v>
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A2,Inventory!$H:$H),2)</f>
+        <v>37837.6</v>
       </c>
       <c r="E2" s="1" t="n">
+        <f aca="false">COUNTIFS(Inventory!$C:$C,A2,Inventory!$I:$I,"&gt;0")</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A2,Inventory!$J:$J),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <f aca="false">COUNTIF(Inventory!$C:$C,A3)</f>
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <f aca="false">SUMIF(Inventory!$C:$C,A3,Inventory!$D:$D)</f>
+        <v>280</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A3,Inventory!$H:$H),2)</f>
+        <v>28397.2</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <f aca="false">COUNTIFS(Inventory!$C:$C,A3,Inventory!$I:$I,"&gt;0")</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A3,Inventory!$J:$J),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <f aca="false">COUNTIF(Inventory!$C:$C,A4)</f>
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <f aca="false">SUMIF(Inventory!$C:$C,A4,Inventory!$D:$D)</f>
+        <v>190</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A4,Inventory!$H:$H),2)</f>
+        <v>75298.1</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <f aca="false">COUNTIFS(Inventory!$C:$C,A4,Inventory!$I:$I,"&gt;0")</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A4,Inventory!$J:$J),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <f aca="false">COUNTIF(Inventory!$C:$C,A5)</f>
         <v>2</v>
       </c>
-      <c r="F2" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>280</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>28397.2</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>190</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>75298.1</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="2" t="n">
+        <f aca="false">SUMIF(Inventory!$C:$C,A5,Inventory!$D:$D)</f>
         <v>115</v>
       </c>
       <c r="D5" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A5,Inventory!$H:$H),2)</f>
         <v>5023.85</v>
       </c>
       <c r="E5" s="1" t="n">
+        <f aca="false">COUNTIFS(Inventory!$C:$C,A5,Inventory!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="F5" s="1" t="n">
+        <f aca="false">ROUND(SUMIF(Inventory!$C:$C,A5,Inventory!$J:$J),2)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>